<commit_message>
101th Commit: Epic One Completed
</commit_message>
<xml_diff>
--- a/EPIC_0001_Platform_Configuration.xlsx
+++ b/EPIC_0001_Platform_Configuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4728EE66-5AB4-4170-967D-7906F75B6EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A971AE26-3D9D-4CEE-971E-8BEA8F8A9D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="Add_Vehicle_Type" sheetId="68" r:id="rId10"/>
     <sheet name="Required_Documents" sheetId="70" r:id="rId11"/>
     <sheet name="Service_Settings" sheetId="71" r:id="rId12"/>
+    <sheet name="DataCleanUpSheet" sheetId="72" r:id="rId13"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="121">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -375,62 +376,6 @@
     <t>Add a new city area with polygon map and verify it appears in the transport services city dropdown in Admin Web</t>
   </si>
   <si>
-    <t>1. Click the dashboard icon
-2. Click the setting menu
-3. Click the city area menu
-4. Wait until the area list heading is visible
-5. Click the add city area button
-6. Wait until the city area add heading is visible
-7. Enter triplicane with timestamp in the area name field
-8. Click the status dropdown
-9. Click the active option
-10. Enter triplicane in the city area search location field
-11. Click the arrow down key on the city area search location field
-12. Click the enter key on the city area search location field
-13. Draw the polygon on the map using coordinates -60;-60, 60;-60, 60;60, -60;60
-14. Click the submit button
-15. Wait until the success message is visible
-16. Click the dashboard icon
-17. Click the transport services menu
-18. Wait until the transport page header is visible
-19. Click the add category button
-20. Click the select city dropdown
-21. Enter the created area name in the filter city field
-22. Verify the area name is displayed in the city dropdown options
-23. Click the close button</t>
-  </si>
-  <si>
-    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-2. Click Setting menu,click,,"web.global.menu.settings"
-3. Click City area menu,click,,"admin.menu.city_area"
-4. Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
-5. Click Add City Area button,click,,"admin.city_area.btn_add"
-6. Wait For City Area heading,wait_until_visible,,"admin.city_area.add_heading"
-7. Enter Area Name,type,triplicane_{timestamp} &gt;&gt; areaName,"admin.city_area.input_name"
-8. Open Status Dropdown,click,,"admin.city_area.dropdown_status"
-9. Select Active,click,,"admin.city_area.select_status_active"
-10. Enter City Area,type,triplicane,"admin.city_area.input_search_location"
-11. wait,1000,,
-12. Select First Option,arrow_down,,"admin.city_area.input_search_location"
-13. Confirm Option,press_enter,,"admin.city_area.input_search_location"
-14. wait,1000,,
-15. Map Polygon,draw polygon,"-60;-60 : 60;-60 : 60;60 : -60;60","//div[@class='ol-layer']//canvas"
-16. Click Submit,click,,"web.global.action.submit"
-17. Wait For Success Message,wait_until_visible,,"web.global.toast.success"
-18. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-19. Click Transport Services,click,,"admin.transport.menu.card"
-20. Wait For Transport Page,wait_until_visible,,"admin.transport.page.header"
-21. Click Add Category,click,,"admin.transport.add_category.btn"
-22. Open Select City Dropdown,click,,"admin.transport.city.dropdown"
-23. Search City Area,type,{areaName},"admin.transport.input_filter_city"
-24. Verify Area in Dropdown,verify,,"admin.transport.city.dynamic_option"
-25. Click close,click,,"web.global.action.close"
-26. wait for data,wait,3000,</t>
-  </si>
-  <si>
-    <t>Access City Area Settings</t>
-  </si>
-  <si>
     <t>SA_RI_57</t>
   </si>
   <si>
@@ -443,82 +388,10 @@
     <t>TC_RG_04_Geo_Fencing</t>
   </si>
   <si>
-    <t>1. Admin is logged in with access to City Area Management.
-2. Service enable for Chennai  City already .
-3. Customer app is logged in and GPS/location is enabled.</t>
-  </si>
-  <si>
     <t>Add a new restricted area and edit it with new name, location in Admin Web</t>
   </si>
   <si>
-    <t>1. Click the dashboard
-2. Click the setting button
-3. Click the geo fencing menu
-4. Click the add restricted area button
-5. Enter chennai airport in the restricted area name field
-6. Click the status toggle button to ON
-7. Enter chennai airport in the search location field
-8. Click the arrow down key on the search location field
-9. Click the enter key on the search location field
-10. Draw the polygon on the map using coordinates -60;-60, 60;-60, 60;60, -60;60
-11. Click the submit button
-12. Enter chennai airport in the area search filter field</t>
-  </si>
-  <si>
     <t>TC_RG_03_City_Area</t>
-  </si>
-  <si>
-    <t>1. Click the dashboard,Click,,"web.global.menu.dashboard"
-2. Click the setting menu,click,"admin.setting.sidebar.menu"
-3. Click the site setting menu,click,"admin.setting.site_setting.sidebar_menu"
-4. Click in clear (X),click,,"admin.settings.btn_clear_driver_algorithm"
-5. Click on driver algorithm,click,,"admin.settings.dropdown_driver_algorithm"
-6. Click the competitive algorithm,click,,"admin.setting.site_settings.driver_algorithm.competitive_algorithm"
-7. Enter 180 seconds,type,180,"admin.settings.input_user_request_timeout"
-8. Click in clear (X),click,,"admin.settings.btn_clear_calculation_method"
-9. wait for,wait,1000
-10. Click the calculate method,click,,"admin.settings.dropdown_calculation_method"
-11. Click the find distance/eta,click,,"admin.setting.site_settings.calculation_for_transport_service.calculation_method"
-12. Click in clear (X),click,,"admin.settings.btn_clear_google_login"
-13. Click the dropdown google,click,,"admin.settings.btn_trigger_google_login"
-14. Click the google ON,click,,"admin.setting.site_settings.social_login.google_login.on"
-15. Click in clear (X),click,,"admin.global.form.btn_clear_provider_subscription"
-16. Click the dropdown driver subscrption,click,,"admin.global.form.btn_trigger_driver_subscription"
-17. Click subscrption button ON,click,,"admin.global.form.dropdown_option_driver_subscription_on"
-18. Click in clear (X),click,,"admin.global.form.btn_clear_cash"
-19. Click the dropdown cash,click,,"admin.global.form.btn_trigger_cash"
-20. Click cash button ON,click,,"admin.setting.site_settings.payments_method.cash.on"
-21.  Click in clear (X),click,,"admin.global.form.btn_clear_wallet"
-22. Click the dropdown wallet,click,,"admin.global.form.btn_trigger_wallet"
-23. Click wallet button ON,click,,"admin.setting.site_settings.wallet.on"
-24. Click in clear (X),click,,"admin.settings.Driver_approval.btn_clear_change_algorithm"
-25. Click the Dropdown,click,,"admin.settings.Driver_approval.btn_trigger_change_algorithm"
-26. Click Driver Approval,click,,"admin.setting.site_settings.account_manual_approvel"
-27. Click in clear (X),click,,"admin.settings.document.btn_clear_change_algorithm"
-28. Click the Dropdown,click,,"admin.settings.document.btn_trigger_change_algorithm"
-29. Click Approval Document,click,,"admin.setting.site_settings.document_manual_approvel"
-30.Click the Dropdown,click,,"admin.settings.document._email_notification_dropdown"
-31.Click On Option,click,,"admin.settings.document._email_notification_option_on"
-32.Click the submit,click,,"admin.settings.btn_submit"</t>
-  </si>
-  <si>
-    <t>1.Click Dashboard,Click,,"web.global.menu.dashboard"
-2.Click Setting Button,click,,"admin.setting.sidebar.menu"
-3.Click Geo Fencing,click,,"admin.setting.geo_fencing.sidebar_menu"
-4.Add Restrict Area,click,,"admin.setting.geo_fencing.add_restricted_area_btn"
-5.Enter Restricted Area Name,type,chennai airport{randomAlpha}&gt;&gt;restrictedArea,"admin.setting.geo_fencing.area_name_input_field"
-6.Click The Status Button On,click,,"admin.setting.geo_fencing.status_toggle_button"
-7. Enter Search Location,type,chennai airport,"admin.city_area.input_search_location"
-8.Wait For Options To Load,wait,3000,
-9. Select First Option,arrow_down,,"admin.city_area.input_search_location"
-10.Confirm Option,press_enter,,"admin.city_area.input_search_location"
-11.Wait For Map To Load,wait,3000,
-12.Map Polygon,draw polygon,"-60;-60 : 60;-60 : 60;60 : -60;60","//div[@class='ol-layer']//canvas"
-13.Wait For Polygon Draw,wait,3000,
-14.Click Submit Button,click,,"admin.setting.geo_fencing.form_submit_button"
-15.Wait For Submit,wait,2000,
-16.Enter Search Area,type,{restrictedArea},"admin.setting.geo_fencing.area_search_filter"
-17.Wait For Load,wait,2000</t>
   </si>
   <si>
     <t>SA_RI_43
@@ -649,42 +522,6 @@
     <t>Verify the admin can manage Home Page Slider and Source Overview successfully</t>
   </si>
   <si>
-    <t>1. Click Dashboard Icon.
-2. Click App Settings.
-3. Click Home Page Slider.
-4. Click Add Button.
-5. Click Select Service field.
-6. Click Select Service.
-7. Enter Image file.
-8. Click Toggle.
-9. Click Submit Button.
-10. Verify Home Page Slider is created successfully.
-11. Click Slider Service Name Grid Search field.
-12. Enter "Auto Ride".
-13. Verify Home Page Slider record is displayed.
-14. Click Edit Icon.
-15. Click Select Service field.
-16. Click Select Service.
-17. Click Uploaded Image field.
-18. Click Banner Image Remove Icon.
-19. Click Status Toggle.
-20. Click Submit Button.
-21. Verify Home Page Slider is updated successfully.
-22. Click Dashboard Icon.
-23. Click App Settings.
-24. Click Source Overview.
-25. Click Add Button.
-26. Click Provider Type field.
-27. Click Provider Type Customer.
-28. Click Source field.
-29. Enter "from facebook".
-30. Click Submit Button.
-31. Verify Source Overview is created successfully.
-32. Click Provider Type Grid Search field.
-33. Enter "customer".
-34. Verify Source Overview record is displayed successfully.</t>
-  </si>
-  <si>
     <t>TC_RG_06_App_Settings</t>
   </si>
   <si>
@@ -705,45 +542,6 @@
   </si>
   <si>
     <t>CF_TC_651</t>
-  </si>
-  <si>
-    <t>1. Click Dashboard.
-2. Click Setting.
-3. Click Panic Call Setting.
-4. Click Add Panic Call Button.
-5. Click Name field.
-6. Enter Name.
-7. Click Name (Tamil) field.
-8. Enter Name (Tamil).
-9. Click Name (Hindi) field.
-10. Enter Name (Hindi).
-11. Click Contact Number field.
-12. Enter Contact Number.
-13. Click Status field.
-14. Click Active Status.
-15. Click Submit Button.
-16. Verify Panic Call record is created successfully.
-17. Click Search Name field.
-18. Enter created Panic Call Name.
-19. Verify Panic Call record is displayed in the search results.</t>
-  </si>
-  <si>
-    <t>1. Click Dashboard,Click,,"web.global.menu.dashboard"
-2. Click Setting,click,,"admin.setting.sidebar.menu"
-3. Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
-4. Click Add panic call button,click,,"admin.setting.panic_call.add_btn"
-5. Enter name,type,police_{randomAlpha}&gt;&gt;policeName,"admin.setting.panic_call.name_input"
-6. Enter name in tamil,type,காவல்துறை,"admin.setting.panic_call.tamil_name_input"
-7. Enter name in hindi,type,पुलिस,"admin.setting.panic_call.hindi_name_input"
-8. Contact number,type,{randomPhone},"admin.setting.panic_call.contact_number"
-9. Select Status button,click,,"admin.setting.panic_call.status_dropdown"
-10. Select Active status,click,,"admin.setting.panic_call.activate_status_dropdown"
-11. Submit button,click,,"web.global.action.submit"
-12. Search name,type,{policeName},"admin.setting.panic_call.search_name"
-13. Wait for data,wait,3000</t>
-  </si>
-  <si>
-    <t>Admin Web user is logged in and Settings module is accessible.</t>
   </si>
   <si>
     <t xml:space="preserve">SA_RI_38
@@ -816,48 +614,6 @@
   </si>
   <si>
     <t>Verify the admin can add a new Transport Service category successfully.</t>
-  </si>
-  <si>
-    <t>a new Transport Service category successfully.
-1. Click Dashboard Icon.
-2. Click Transport Services Menu.
-3. Verify Transport Services page is displayed.
-4. Click Add Category.
-5. Click Service Name field.
-6. Enter Service Name.
-7. Click Service Name (Arabic) field.
-8. Enter Service Name (Arabic).
-9. Click Slug field.
-10. Enter Slug.
-11. Click Transport Service Image field.
-12. Enter Transport Service Image.
-13. Click Status Dropdown.
-14. Click Activate Status.
-15. Click Select City Dropdown.
-16. Click City option.
-17. Click Submit Button.
-18. Verify Transport Service category is created successfully.
-19. Click Back Button.
-20. Verify Transport Services listing page is displayed.</t>
-  </si>
-  <si>
-    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
-2. Click Transports Services Menu,click,, "admin.transport.menu.card"
-3.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
-4.Click  Add Category,click,, "admin.transport.add_category.btn"
-5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "admin.transport.name.input"
-6.Enter Service Name Arabic, type, رحلة بالحافلة, "admin.transport.name_ar.input"
-7.Enter Slug, type, Bus Ride, "admin.transport.slug.input"
-8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "admin.transport.image.file"
-9.wait,2000,,
-10.Open status Dropdown,click,, "admin.transport.status.dropdown"
-11.Select Activate,click,, "admin.transport.status.activate_option"
-12.Open Select City Dropdown,click,, "admin.transport.city.dropdown"
-13.Select {areaName},click,, "admin.transport.city.dynamic_option"
-14.Click  Submit,click,, "web.global.action.submit"
-15.Wait Till Sucess, wait_until_visible, , "web.global.toast.info"
-16.wait,2000,,
-17.Click  back,click,, "admin.transport.back.btn"</t>
   </si>
   <si>
     <t>Admin Web user is logged in, Transport Services module is accessible, and at least one City is available for selection.</t>
@@ -1147,6 +903,578 @@
 26.wait for popup,wait,2000,</t>
   </si>
   <si>
+    <t>1. Click the dashboard,Click,,"web.global.menu.dashboard"
+2. Click the setting menu,click,"admin.setting.sidebar.menu"
+3. Click the site setting menu,click,"admin.setting.site_setting.sidebar_menu"
+4. Click in clear (X),click,,"admin.settings.btn_clear_driver_algorithm"
+5. Click on driver algorithm,click,,"admin.settings.dropdown_driver_algorithm"
+6. Click the competitive algorithm,click,,"admin.setting.site_settings.driver_algorithm.competitive_algorithm"
+7. Enter 180 seconds,type,180,"admin.settings.input_user_request_timeout"
+8. Click in clear (X),click,,"admin.settings.btn_clear_calculation_method"
+9. wait for,wait,1000
+10. Click the calculate method,click,,"admin.settings.dropdown_calculation_method"
+11. Click the find distance/eta,click,,"admin.setting.site_settings.calculation_for_transport_service.calculation_method"
+12. Click in clear (X),click,,"admin.settings.btn_clear_google_login"
+13. Click the dropdown google,click,,"admin.settings.btn_trigger_google_login"
+14. Click the google ON,click,,"admin.setting.site_settings.social_login.google_login.on"
+15. Click in clear (X),click,,"admin.global.form.btn_clear_provider_subscription"
+16. Click the dropdown driver subscrption,click,,"admin.global.form.btn_trigger_driver_subscription"
+17. Click subscrption button ON,click,,"admin.global.form.dropdown_option_driver_subscription_on"
+18. Click in clear (X),click,,"admin.global.form.btn_clear_cash"
+19. Click the dropdown cash,click,,"admin.global.form.btn_trigger_cash"
+20. Click cash button ON,click,,"admin.setting.site_settings.payments_method.cash.on"
+21.  Click in clear (X),click,,"admin.global.form.btn_clear_wallet"
+22. Click the dropdown wallet,click,,"admin.global.form.btn_trigger_wallet"
+23. Click wallet button ON,click,,"admin.setting.site_settings.wallet.on"
+24. Click in clear (X),click,,"admin.settings.Driver_approval.btn_clear_change_algorithm"
+25. Click the Dropdown,click,,"admin.settings.Driver_approval.btn_trigger_change_algorithm"
+26. Click Driver Approval,click,,"admin.setting.site_settings.account_manual_approvel"
+27. Click in clear (X),click,,"admin.settings.document.btn_clear_change_algorithm"
+28. Click the Dropdown,click,,"admin.settings.document.btn_trigger_change_algorithm"
+29. Click Approval Document,click,,"admin.setting.site_settings.document_manual_approvel"
+30.Click the Dropdown,click,,"admin.settings.document._email_notification_dropdown"
+31.Click On Option,click,,"admin.settings.document._email_notification_option_on"
+32.Click the submit,click,,"admin.settings.btn_submit"
+33.Wait For Submit,wait,2000,</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Setting menu,click,,"web.global.menu.settings"
+3. Click City area menu,click,,"admin.menu.city_area"
+4. Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
+5. Click Add City Area button,click,,"admin.city_area.btn_add"
+6. Wait For City Area heading,wait_until_visible,,"admin.city_area.add_heading"
+7. Enter Area Name,type,triplicane_{timestamp} &gt;&gt; areaName,"admin.city_area.input_name"
+8. Open Status Dropdown,click,,"admin.city_area.dropdown_status"
+9. Select Active,click,,"admin.city_area.select_status_active"
+10. Enter City Area,type,triplicane,"admin.city_area.input_search_location"
+11. wait,1000,,
+12. Select First Option,arrow_down,,"admin.city_area.input_search_location"
+13. Confirm Option,press_enter,,"admin.city_area.input_search_location"
+14. wait,1000,,
+15. Map Polygon,draw polygon,"-60;-60 : 60;-60 : 60;60 : -60;60","//div[@class='ol-layer']//canvas"
+16. Click Submit,click,,"web.global.action.submit"
+17. Wait For Success Message,wait_until_visible,,"web.global.toast.success"
+18. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+19. Click Transport Services,click,,"admin.transport.menu.card"
+20. Wait For Transport Page,wait_until_visible,,"admin.transport.page.header"
+21. Click Add Category,click,,"admin.transport.add_category.btn"
+22. Open Select City Dropdown,click,,"admin.transport.city.dropdown"
+23. Search City Area,type,{areaName},"admin.transport.input_filter_city"
+24. Verify Area in Dropdown,verify,,"admin.transport.city.dynamic_option"
+25. Click close,click,,"web.global.action.close"
+26. wait for data,wait,2000,
+27.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+28. Click Setting menu,click,,"web.global.menu.settings"
+29. Click City admin menu,click,,"admin.menu.city_admin"
+30. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
+31. Click Add City Admin button,click,,"admin.city_admin.btn_add"
+32. Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
+33. Select {areaName},click,,"admin.city_admin.select_dynamic_option"
+34. Verify Selection,verify,,"admin.city_admin.verify_dropdown_value"
+35.Wait For Verify,wait,2000,
+36.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+37.Click Setting menu,click,,"web.global.menu.settings"
+38.Click City area menu,click,,"admin.menu.city_area"
+39.Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
+40.Serch Created Area,type,{areaName},"admin.city_area.area_filter_input"
+41.Wait For Load,wait,1000,
+42.Click City Area Edit,click,,"admin.city_area.edit_button"
+43.Open Status Dropdown,click,,"admin.city_area.dropdown_active_status"
+44.Select Inactive,click,,"admin.city_area.select_status_inactive"
+45.Click Submit,click,,"web.global.action.submit"
+46.Wait For Submit,2000,</t>
+  </si>
+  <si>
+    <t>1. Log into the Super Admin Web Portal and click the Dashboard Icon on the sidebar menu.
+2. Click on the Settings Menu option.
+3. Click on the City Area sub-menu link.
+4. Verify that the City Area management list heading displays correctly.
+5. Click the "Add City Area" button.
+6. Verify the "Add City Area" page/modal heading displays.
+7. Enter a unique Area Name (e.g., "triplicane_&lt;timestamp&gt;").
+8. Click the Status dropdown menu.
+9. Select "Active" status from the options.
+10. Type "triplicane" into the search location input field.
+11. Press the Down Arrow key on the keyboard to highlight the first location suggestion.
+12.Press Enter to select and confirm the location.
+13. Draw a polygon boundary on the map canvas using the specified coordinates (-60;-60 : 60;-60 : 60;60 : -60;60).
+14.Click the Submit button to save the new City Area.
+15.Verify that the "Success" toast message appears.
+16.Click the Dashboard Icon on the sidebar menu.
+17.Click the Transport Services card/menu item.
+18.Verify that the Transport Services page header displays.
+19.Click the "Add Category" button.
+20.Click the Select City dropdown.
+21.Type the newly created area name into the city filter search input.
+22.Verify that the newly created City Area appears dynamically in the dropdown list.
+23.Click the Close/Cancel button on the modal.
+24.Click the Dashboard Icon on the sidebar menu.
+25.Click on the Settings Menu option.
+26.Click on the City Admin sub-menu link.
+27.Verify that the City Admin management list heading displays.
+28.Click the "Add City Admin" button.
+29.Click the Select City dropdown.
+30.Select the created City Area from the dynamic option list.
+31.Verify that the selected area is correctly displayed in the dropdown selection field.
+32.Click the Dashboard Icon on the sidebar menu.
+33.Click on the Settings Menu option.
+34.Click on the City Area sub-menu link.
+35.Verify that the City Area management list heading displays.
+36.Type the created area name into the Area Filter search input field.
+37.Click the Edit button for the filtered City Area.
+38. Click the Status dropdown menu.
+39. Select "Inactive" status from the options.
+40. Click the Submit button to save the updated status.</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard,Click,,"web.global.menu.dashboard"
+2.Click Setting Button,click,,"admin.setting.sidebar.menu"
+3.Click Geo Fencing,click,,"admin.setting.geo_fencing.sidebar_menu"
+4.Add Restrict Area,click,,"admin.setting.geo_fencing.add_restricted_area_btn"
+5.Enter Restricted Area Name,type,chennai airport{randomAlpha}&gt;&gt;restrictedArea,"admin.setting.geo_fencing.area_name_input_field"
+6.Click The Status Button On,click,,"admin.setting.geo_fencing.status_toggle_button"
+7. Enter Search Location,type,chennai airport,"admin.city_area.input_search_location"
+8.Wait For Options To Load,wait,3000,
+9. Select First Option,arrow_down,,"admin.city_area.input_search_location"
+10.Confirm Option,press_enter,,"admin.city_area.input_search_location"
+11.Wait For Map To Load,wait,3000,
+12.Map Polygon,draw polygon,"-60;-60 : 60;-60 : 60;60 : -60;60","//div[@class='ol-layer']//canvas"
+13.Wait For Polygon Draw,wait,3000,
+14.Click Submit Button,click,,"admin.setting.geo_fencing.form_submit_button"
+15.Wait For Submit,wait,2000,
+16.Enter Search Area,type,{restrictedArea},"admin.setting.geo_fencing.area_search_filter"
+17.Wait For Geo Fenced Area To Load,wait,2000
+18.Delete Geo Fenced Area,click,,"admin.setting.geo_fencing.delete_button"
+19.Cofirm Deletion,click,,"admin.setting.geo_fencing.confirm_delete_button"
+20.Wait For Deletion,wait,2000,</t>
+  </si>
+  <si>
+    <t>1. Click the dashboard
+2. Click the setting button
+3. Click the geo fencing menu
+4. Click the add restricted area button
+5. Enter chennai airport in the restricted area name field
+6. Click the status toggle button to ON
+7. Enter chennai airport in the search location field
+8. Click the arrow down key on the search location field
+9. Click the enter key on the search location field
+10. Draw the polygon on the map using coordinates -60;-60, 60;-60, 60;60, -60;60
+11. Click the submit button
+12. Enter chennai airport in the area search filter field
+13.Delete The Geo Fenced Area</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click app settings,click,,"admin.app_settings"
+3. Click home page slider,click,,"admin.app_settings.home_page_slider"
+4. Click add button,click,,"admin.app_settings.home_page_slider.add"
+5. Click select service field,click,,"admin.app_settings.home_page_slider.select_service"
+6. Click select service,click,,"admin.app_settings.home_page_slider.select_taxi"
+7. Upload image,upload file,"src/main/resources/test-data/audi.jpg","admin.app_settings.home_page_slider.upload_image"
+8. Click toggle,click,,"admin.app_settings.home_page_slider.toggle"
+9. Click submit button,click,,"admin.app_settings.home_page_slider.submit"
+10.Wait For Submit,wait,2000,
+11.Type Taxi Ride In Service Name Grid Search,type ,Taxi Ride,"admin.app_settings.home_page_slider.gride_search_Slider_service_name"
+12.Delete Page Slider,click,,"admin.app_settings.home_page_slider.delete_icon"
+13.Cofirm Slider Delete,click,,"admin.app_settings.home_page_slider.delete_yes"
+14.Wait For Popup To Vanish,wait,2000,
+15.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+16.Click app settings,click,,"admin.app_settings"
+17.Click source overview,click,,"admin.setting.source_overview"
+18.Click add button,click,,"admin.setting.source_overview.add_button"
+19.Click provider type,click,,"admin.setting.source_overview.provider_type"
+20.Click provider type customer,click,,"admin.setting.source_overview.provider_type_customer" 
+21.Click source field,click,,"admin.setting.source_overview.source_field"
+22.Type source field,type ,From Facebook,"admin.setting.source_overview.source_field"
+23.Click submit button,click,,"web.global.action.submit"
+24.Wait For Submit,wait,2000,
+25.Click Source  Grid Search,click,,"admin.setting.source_overview.source_filter_input"
+26.Type source field,type ,From Facebook,"admin.setting.source_overview.source_filter_input"
+27.Wait To Load,wait,1000,
+28.Delete Source Overview,click,,"admin.app_settings.source_overview.delete_icon"
+29.Cofirm Source Overview Delete,click,,"admin.app_settings.source_overview.delete_yes"
+30.Wait For Delete,wait,2000,</t>
+  </si>
+  <si>
+    <t>Super Admin Is logged In And Has Acces To Add City Area Settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin is logged in with access to Geo Fencing Management.
+</t>
+  </si>
+  <si>
+    <t>Admin Web user is logged in and Panic Call module is accessible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Log into the Super Admin Web Portal and click the Dashboard Icon on the sidebar menu.
+2. Click on the App Settings menu option.
+3. Click on the Home Page Slider sub-menu link.
+4. Click the "Add" button to create a new slider configuration.
+5. Click the Select Service dropdown field.
+6. Select "Taxi" service from the dropdown list.
+7. Upload a slider banner image file from local resources ("src/main/resources/test-data/audi.jpg").
+8. Click the Status Toggle switch to enable the slider.
+9. Click the Submit button to save the new home page slider.
+10. Type "Taxi Ride" into the Slider Service Name grid search filter input.
+11. Click the Delete icon for the filtered slider record.
+12. Click "Yes" on the confirmation pop-up to confirm slider deletion.
+13. Wait 2 seconds for the deletion modal to dismiss.
+14. Click the Dashboard Icon on the sidebar menu.
+15. Click on the App Settings menu option.
+16. Click on the Source Overview sub-menu link.
+17. Click the "Add" button to add a new source overview entry.
+18. Click the Provider Type dropdown field.
+19. Select "Customer" as the provider type option.
+20. Click the Source Field input box.
+21. Type "From Facebook" into the Source Field.
+22. Click the Submit button to save the new source overview entry.
+23. Click the Source Grid Search filter input field.
+24. Type "From Facebook" into the grid filter search box.
+25. Click the Delete icon for the filtered source overview record.
+26. Click "Yes" on the confirmation pop-up to confirm deletion.
+</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard,Click,,"web.global.menu.dashboard"
+2. Click Setting,click,,"admin.setting.sidebar.menu"
+3. Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
+4. Click Add panic call button,click,,"admin.setting.panic_call.add_btn"
+5. Enter name,type,police_{randomAlpha}&gt;&gt;policeName,"admin.setting.panic_call.name_input"
+6. Enter name in tamil,type,காவல்துறை,"admin.setting.panic_call.tamil_name_input"
+7. Enter name in hindi,type,पुलिस,"admin.setting.panic_call.hindi_name_input"
+8. Contact number,type,{randomPhone},"admin.setting.panic_call.contact_number"
+9. Select Status button,click,,"admin.setting.panic_call.status_dropdown"
+10. Select Active status,click,,"admin.setting.panic_call.activate_status_dropdown"
+11. Submit button,click,,"web.global.action.submit"
+12. Search name,type,{policeName},"admin.setting.panic_call.search_name"
+13.Wait For Load,wait,1000,
+14.Delete Panic Call Delete,click,,"admin.setting.panic_call.delete_btn"
+15.Confirm Delete,click,,"admin.setting.panic_call.confirm_delete_btn"
+16. Wait For Delete,wait,2000,</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard.
+2. Click Setting.
+3. Click Panic Call Setting.
+4. Click Add Panic Call Button.
+5. Click Name field.
+6. Enter Name.
+7. Click Name (Tamil) field.
+8. Enter Name (Tamil).
+9. Click Name (Hindi) field.
+10. Enter Name (Hindi).
+11. Click Contact Number field.
+12. Enter Contact Number.
+13. Click Status field.
+14. Click Active Status.
+15. Click Submit Button.
+16. Verify Panic Call record is created successfully.
+17. Click Search Name field.
+18. Enter created Panic Call Name.
+19. Verify Panic Call record is displayed in the search results.
+20.Delete The Displayed Panic Call</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2. Click Transports Services Menu,click,, "admin.transport.menu.card"
+3.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+4.Click  Add Category,click,, "admin.transport.add_category.btn"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "admin.transport.name.input"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "admin.transport.name_ar.input"
+7.Enter Slug, type, Bus Ride, "admin.transport.slug.input"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "admin.transport.image.file"
+9.wait,2000,,
+10.Open status Dropdown,click,, "admin.transport.status.dropdown"
+11.Select Activate,click,, "admin.transport.status.activate_option"
+12.Open Select City Dropdown,click,, "admin.transport.city.dropdown"
+13.Select City Area,click,,"admin.transport.city.dynamic_option_regression_city_area"
+14.Click  Submit,click,, "web.global.action.submit"
+15.Wait Till Sucess, wait_until_visible, , "web.global.toast.info"
+16.Wait To Load,wait,2000,
+17.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+18.Click Transports Services Menu,click,, "admin.transport.menu.card"
+19.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+20.Select Transport Service Name,type,{transportName},"admin.transport.grid.name_filter"
+21.Wait For Load,wait,2000,
+22.Click Edit,click,,"admin.transport.edit_btn"
+23.Scroll Transport From,tab,5,"admin.transport.name.input"
+24.Open status Dropdown,click,, "admin.transport.status.dropdown"
+25.Select Deactivate,click,, "admin.transport.status.deactivate_option"
+26.Click  Submit,click,, "web.global.action.submit"
+27.Wait For Update,wait,2000,
+28.Click  back,click,, "admin.transport.back.btn"</t>
+  </si>
+  <si>
+    <t>a new Transport Service category successfully.
+1. Click Dashboard Icon.
+2. Click Transport Services Menu.
+3. Verify Transport Services page is displayed.
+4. Click Add Category.
+5. Click Service Name field.
+6. Enter Service Name.
+7. Click Service Name (Arabic) field.
+8. Enter Service Name (Arabic).
+9. Click Slug field.
+10. Enter Slug.
+11. Click Transport Service Image field.
+12. Enter Transport Service Image.
+13. Click Status Dropdown.
+14. Click Activate Status.
+15. Click Select City Dropdown.
+16. Click City option.
+17. Click Submit Button.
+18. Verify Transport Service category is created successfully.
+19. Click Back Button.
+20. Verify Transport Services listing page is displayed.
+21.Search For The Created Transport Service in Service search box
+22.Click Edit Button
+23.Deactivate the transport service
+24.Click Submit</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2.Click Transports Services Menu,click,, "admin.transport.menu.card"
+3.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
+4.Click Home Icon ,click,, "admin.transport.home.icon"
+5.Click Settings ,click,, "admin.transport.menu.settings"
+6.Click Vehicle Type,click,, "admin.transport.settings.vehicle_type"
+7.Click Add Vehicle Type,click,, "admin.transport.vehicle.add_type.btn"
+8.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "admin.transport.vehicle.name.input"
+9.Enter Base Fare, type, 150, "admin.transport.vehicle.base_fare.input"
+10.Enter Base Fare Max Kilometer, type, 10, "admin.transport.vehicle.base_km.input"
+11.Open Extra Distance Fare Dropdown,click,, "admin.transport.vehicle.extra_fare_type.dropdown"
+12.Select Amount,click,, "admin.transport.status.amount_option"
+13.Enter Extra Distance Fare , type, 10, "admin.transport.vehicle.extra_fare.input"
+14.Enter Free Waiting Time , type, 10, "admin.transport.vehicle.waiting_free.input"
+15.Open Waiting Charge Dropdown,click,, "admin.transport.vehicle.waiting_type.dropdown"
+16.Select Amount,click,, "admin.transport.status.amount_option"
+17.Enter Waiting Rate , type, 10, "admin.transport.vehicle.waiting_rate.input"
+18.Enter Included Trip Waiting , type, 10, "admin.transport.vehicle.trip_waiting_free.input"
+19.Open Trip Waiting Charge Dropdown,click,, "admin.transport.vehicle.trip_waiting_type.dropdown"
+20.Select Amount,click,, "admin.transport.status.amount_option"
+21.Enter Trip Waiting Rate , type,50, "admin.transport.vehicle.trip_waiting_rate.input"
+22.Enter Free Pickup Distance , type,5, "admin.transport.vehicle.pickup_free.input"
+23.Open Pickup Charge Dropdown,click,, "admin.transport.vehicle.pickup_type.dropdown"
+24.Select Amount,click,, "admin.transport.status.amount_option"
+25.Enter Pickup Fee, type,50, "admin.transport.vehicle.pickup_fee.input"
+26.Open Customer Fee  Dropdown,click,, "admin.transport.vehicle.customer_type.dropdown"
+27.Select Amount,click,, "admin.transport.status.amount_option"
+28.Enter Customer Fee, type,50, "admin.transport.vehicle.customer_fee.input"
+29.Open Customer GST  Dropdown,click,, "admin.transport.vehicle.customer_gst_type.dropdown"
+30.Select Amount,click,, "admin.transport.status.amount_option"
+31.Enter  GST amount, type,50, "admin.transport.vehicle.customer_gst.input"
+32.Open Driver Fee  Dropdown,click,, "admin.transport.vehicle.driver_type.dropdown"
+33.Select Amount,click,, "admin.transport.status.amount_option"
+34.Enter  Driver Fee, type,50, "admin.transport.vehicle.driver_fee.input"
+35.Open Driver GST  Dropdown,click,, "admin.transport.vehicle.driver_gst_type.dropdown"
+36.Select Amount,click,, "admin.transport.status.amount_option"
+37.Enter Driver Gst,type,50, "admin.transport.vehicle.driver_gst.input"
+38.Open Status Dropdown,click,, "admin.transport.vehicle.status.dropdown"
+39.Select Active,click,, "admin.transport.status.active_option"
+40.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "admin.transport.vehicle.image.file"
+41.Enter Notifiacation,type,50, "admin.transport.vehicle.notify_km.input"
+42.Enter Driver Request ETA,type,50, "admin.transport.vehicle.eta_limit.input"
+43.Enter Driver Request KM,type,50, "admin.transport.vehicle.km_limit.input"
+44.Enter Package Idle Free Time,type,30,"admin.transport.vehicle.package_idle_free_time"
+45.Enter Package Idle Time Fee,type,50,"admin.transport.vehicle.package_idle_time_fee"
+46.Open Night Charge Timing Status Dropdown,click,, "admin.transport.night.status.dropdown"
+47.Select Active,click,, "admin.transport.status.active_option"
+48.Click Surcharge Time Checkbox, click, , "admin.transport.night.everyday.checkbox"
+49.Enter From Time, type, 100000AM, "admin.transport.night.from_time.input"
+50.Enter To Time, type, 220000PM, "admin.transport.night.to_time.input"
+51.Open  Dropdown,click,, "admin.transport.night.type.dropdown"
+52.Select Amount,click,, "admin.transport.status.amount_option"
+53.Enter  Price, type,50, "admin.transport.night.price.input"
+54.Click  Submit,click,, "web.global.action.submit"
+55.Wait For Sucess,wait_until_visible, , "web.global.toast.info"
+56.Wait For Popup,wait,3000,</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard,Click,,"web.global.menu.dashboard"
+2.Click Transport Service,Click,,"admin.transport.menu.card"
+3.Click Search Box,click,,"admin.transport.search.input_box"
+4.Enter Services,type,{transportName},"admin.transport.search.input_box"
+5.Click Home Icon,Click,,"admin.transport.home.icon"
+6.Click Settings ,click,,"admin.transport.menu.settings"
+7.Click Requirment Document ,click,,"admin.transport.docs.menu_item"
+8.Click Add Document ,click,,"admin.transport.docs.add.btn"
+9.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "admin.transport.docs.name.input"
+10.Open status Dropdown,click,,"admin.transport.docs.status.dropdown"
+11.Select Active,click,,"admin.transport.status.active_option"
+12.Click Document Expiry ,click,,"admin.transport.docs.expiry.checkbox"
+13.Click Mandatory Document ,click,,"admin.transport.docs.mandatory.checkbox"
+14.Click  Require Proof Number,click,,"admin.transport.docs.proof_no.checkbox"
+15.Enter Display Order, type, 10, "admin.transport.docs.order.input"
+16.Click Submit ,click,,"web.global.action.submit"
+17.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+18.Filter Document List,type,{documentName}, "admin.transport.docs.grid.name_filter"
+19.wait for data,wait,1000,</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard,Click,,"web.global.menu.dashboard"
+2.Click Transport Service,Click,,"admin.transport.menu.card"
+3.Click Search Box,click,,"admin.transport.search.input_box"
+4.Enter Services,type,{transportName},"admin.transport.search.input_box"
+5.Click Home Icon,Click,,"admin.transport.home.icon"
+6.Click Settings ,click,, "admin.transport.menu.settings"
+7.Click Service Settings ,click,, "admin.transport.rules.menu_item"
+8.Enter Driver Accept Timeout, type, 60, "admin.transport.rules.timeout.input"
+9.Enter Driver Serach Radius, type, 50, "admin.transport.rules.radius.input"
+10.Click Submit ,click,, "web.global.action.submit"
+11.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
+12.wait for Notification,wait,1000,</t>
+  </si>
+  <si>
+    <t>Pre-production</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
+  <si>
+    <t>TC_SA_29_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>This test phase ensures the long-term stability and performance of the QA environment by executing a systematic Automated Data Cleanup strategy. Leveraging localized SQL Hooks with built-in safety firewalls, the workflow identifies and removes dynamically generated test artifacts—including unique City Areas, Provider profiles, and administrative accounts—created during the regression suite. By targeting specific records using variable-driven WHERE clauses, the script maintains database referential integrity, prevents record duplication in subsequent runs, and ensures the test environment remains in a pristine, 'ready-state' for continuous integration</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CRITICAL SYSTEM WARNING: DATABASE INTEGRITY PROTOCOL</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-----------------------------------------</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">This sheet contains SQL Hooks that execute directly against the we1 Production/Staging database. DO NOT modify the SQL syntax, remove variable placeholders (e.g., {areaName}), or edit the WHERE clauses.
+Unauthorized changes may result in irreversible data loss or database corruption. If modifications are required, please contact the Automation Lead or the Database Administrator.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSWORD TO EDIT SHEET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> :eit6190
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.
+RunSheet: SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
+2.Remove  Document Created,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
+3..Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
+4.Remove  Transport Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
+</t>
+  </si>
+  <si>
+    <t>SA_TS_XX</t>
+  </si>
+  <si>
+    <t>Clean The Test Data Created During Test Run Of Epic One</t>
+  </si>
+  <si>
+    <t>TC_RG_13_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>No Manual Test Cases Since this is a data cleanup sheet after test execution of epic one</t>
+  </si>
+  <si>
     <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 2. Click Page list menu,click,,"admin.page_list"
 3. Click customer app support,click,,"admin.page_list.customer_app_support"
@@ -1169,7 +1497,7 @@
 20.Click Arabic Field,click,,"admin.page_list.common.name_arabic.input"
 21. wait for loading,wait,5000,
 22. Click privacy policy,click,,"admin.page_list.customer_app_support.privacy_policy"
-23. Clear the name field in arabic,clear,,"admin.page_list.common.name_arabic.input"
+23. Clear the name field in arabic,clear,,"admin.page_list.common.name_arabic_privacy_policy.input"
 24. Enter the Name (Arabic),Type,اتصل,"admin.page_list.common.name_arabic_privacy_policy.input"
 25. Clear the name field in tamil,clear,,"admin.page_list.common.name_tamil.input"
 26. Enter the Name (Tamil),Type,தனியுரிமைக் கொள்கை,"admin.page_list.common.name_tamil.input"
@@ -1249,71 +1577,12 @@
 100.Click the Submit button,click,,"web.global.action.submit.button"
 101.wait for loading,wait,5000,</t>
   </si>
-  <si>
-    <t>1.Click Dashboard,Click,,"web.global.menu.dashboard"
-2.Click Transport Service,Click,,"admin.transport.menu.card"
-3.Click Search Box,click,,"admin.transport.search.input_box"
-4.Enter Services,type,Auto Ride,"admin.transport.search.input_box"
-5.Click Home Icon,Click,,"admin.transport.home.icon"
-6.Click Settings ,click,,"admin.transport.menu.settings"
-7.Click Requirment Document ,click,,"admin.transport.docs.menu_item"
-8.Click Add Document ,click,,"admin.transport.docs.add.btn"
-9.Enter Name, type, documet{randomAlpha}&gt;&gt; documentName, "admin.transport.docs.name.input"
-10.Open status Dropdown,click,,"admin.transport.docs.status.dropdown"
-11.Select Active,click,,"admin.transport.status.active_option"
-12.Click Document Expiry ,click,,"admin.transport.docs.expiry.checkbox"
-13.Click Mandatory Document ,click,,"admin.transport.docs.mandatory.checkbox"
-14.Click  Require Proof Number,click,,"admin.transport.docs.proof_no.checkbox"
-15.Enter Display Order, type, 10, "admin.transport.docs.order.input"
-16.Click Submit ,click,,"web.global.action.submit"
-17.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
-18.Filter Document List,type,{documentName}, "admin.transport.docs.grid.name_filter"
-19.wait for data,wait,1000,</t>
-  </si>
-  <si>
-    <t>1.Click Dashboard,Click,,"web.global.menu.dashboard"
-2.Click Transport Service,Click,,"admin.transport.menu.card"
-3.Click Search Box,click,,"admin.transport.search.input_box"
-4.Enter Services,type,Auto Ride,"admin.transport.search.input_box"
-5.Click Home Icon,Click,,"admin.transport.home.icon"
-6.Click Settings ,click,, "admin.transport.menu.settings"
-7.Click Service Settings ,click,, "admin.transport.rules.menu_item"
-8.Enter Driver Accept Timeout, type, 60, "admin.transport.rules.timeout.input"
-9.Enter Driver Serach Radius, type, 50, "admin.transport.rules.radius.input"
-10.Click Submit ,click,, "web.global.action.submit"
-11.Wait For Sucess, wait_until_visible, , "web.global.toast.info"
-12.wait for Notification,wait,1000,</t>
-  </si>
-  <si>
-    <t>1.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-2. Click app settings,click,,"admin.app_settings"
-3. Click home page slider,click,,"admin.app_settings.home_page_slider"
-4. Click add button,click,,"admin.app_settings.home_page_slider.add"
-5. Click select service field,click,,"admin.app_settings.home_page_slider.select_service"
-6. Click select service,click,,"admin.app_settings.home_page_slider.select"
-7. Upload image,upload file,"src/main/resources/test-data/audi.jpg","admin.app_settings.home_page_slider.upload_image"
-8. Click toggle,click,,"admin.app_settings.home_page_slider.toggle"
-9. Click submit button,click,,"admin.app_settings.home_page_slider.submit"
-10. Type auto ride service name gride search,type ,Auto Ride,"admin.app_settings.home_page_slider.gride_search_Slider_service_name"
-18. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-19. Click app settings,click,,"admin.app_settings"
-20. Click source overview,click,,"admin.setting.source_overview"
-21. Click add button,click,,"admin.setting.source_overview.add_button"
-22. Click provider type,click,,"admin.setting.source_overview.provider_type"
-23. Click provider type customer,click,,"admin.setting.source_overview.provider_type_customer"
-24. Click source field,click,,"admin.setting.source_overview.source_field"
-25. Type source field,type ,from facebook,"admin.setting.source_overview.source_field"
-26. Click submit button,click,,"web.global.action.submit"
-27. Click provide type gride search,click,,"admin.setting.source_overview.provider_type_gride_search"
-28. Type source field,type ,customer,"admin.setting.source_overview.provider_type_gride_search"
-29. Wait for data,wait,2000,</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1333,6 +1602,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1364,7 +1641,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1377,6 +1654,16 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1799,33 +2086,35 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J2" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -1897,31 +2186,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -1995,31 +2284,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2039,6 +2328,94 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F212A7B3-E2B5-43F7-B627-2EE6125B3067}">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" customWidth="1"/>
+    <col min="5" max="6" width="34.109375" customWidth="1"/>
+    <col min="7" max="7" width="69.33203125" customWidth="1"/>
+    <col min="8" max="8" width="31.77734375" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="8"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2111,7 +2488,7 @@
         <v>24</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2200,22 +2577,22 @@
         <v>31</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2289,31 +2666,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>97</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2387,31 +2764,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2485,31 +2862,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2583,31 +2960,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>65</v>
+        <v>104</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2681,31 +3058,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2779,31 +3156,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="J2" s="2"/>
     </row>

</xml_diff>

<commit_message>
102th Commit: Epic One Updated
</commit_message>
<xml_diff>
--- a/EPIC_0001_Platform_Configuration.xlsx
+++ b/EPIC_0001_Platform_Configuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A971AE26-3D9D-4CEE-971E-8BEA8F8A9D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E67BB8-CAC1-47BD-BA87-21E8185578DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -901,41 +901,6 @@
 24.Click Deactive Button,click,,"web.global.report_issue.faq.deactivate.button"
 25.Click Active Button,click,,"web.global.report_issue.faq.activate.button"
 26.wait for popup,wait,2000,</t>
-  </si>
-  <si>
-    <t>1. Click the dashboard,Click,,"web.global.menu.dashboard"
-2. Click the setting menu,click,"admin.setting.sidebar.menu"
-3. Click the site setting menu,click,"admin.setting.site_setting.sidebar_menu"
-4. Click in clear (X),click,,"admin.settings.btn_clear_driver_algorithm"
-5. Click on driver algorithm,click,,"admin.settings.dropdown_driver_algorithm"
-6. Click the competitive algorithm,click,,"admin.setting.site_settings.driver_algorithm.competitive_algorithm"
-7. Enter 180 seconds,type,180,"admin.settings.input_user_request_timeout"
-8. Click in clear (X),click,,"admin.settings.btn_clear_calculation_method"
-9. wait for,wait,1000
-10. Click the calculate method,click,,"admin.settings.dropdown_calculation_method"
-11. Click the find distance/eta,click,,"admin.setting.site_settings.calculation_for_transport_service.calculation_method"
-12. Click in clear (X),click,,"admin.settings.btn_clear_google_login"
-13. Click the dropdown google,click,,"admin.settings.btn_trigger_google_login"
-14. Click the google ON,click,,"admin.setting.site_settings.social_login.google_login.on"
-15. Click in clear (X),click,,"admin.global.form.btn_clear_provider_subscription"
-16. Click the dropdown driver subscrption,click,,"admin.global.form.btn_trigger_driver_subscription"
-17. Click subscrption button ON,click,,"admin.global.form.dropdown_option_driver_subscription_on"
-18. Click in clear (X),click,,"admin.global.form.btn_clear_cash"
-19. Click the dropdown cash,click,,"admin.global.form.btn_trigger_cash"
-20. Click cash button ON,click,,"admin.setting.site_settings.payments_method.cash.on"
-21.  Click in clear (X),click,,"admin.global.form.btn_clear_wallet"
-22. Click the dropdown wallet,click,,"admin.global.form.btn_trigger_wallet"
-23. Click wallet button ON,click,,"admin.setting.site_settings.wallet.on"
-24. Click in clear (X),click,,"admin.settings.Driver_approval.btn_clear_change_algorithm"
-25. Click the Dropdown,click,,"admin.settings.Driver_approval.btn_trigger_change_algorithm"
-26. Click Driver Approval,click,,"admin.setting.site_settings.account_manual_approvel"
-27. Click in clear (X),click,,"admin.settings.document.btn_clear_change_algorithm"
-28. Click the Dropdown,click,,"admin.settings.document.btn_trigger_change_algorithm"
-29. Click Approval Document,click,,"admin.setting.site_settings.document_manual_approvel"
-30.Click the Dropdown,click,,"admin.settings.document._email_notification_dropdown"
-31.Click On Option,click,,"admin.settings.document._email_notification_option_on"
-32.Click the submit,click,,"admin.settings.btn_submit"
-33.Wait For Submit,wait,2000,</t>
   </si>
   <si>
     <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
@@ -1576,6 +1541,43 @@
 99. Enter the Name (Tamil),Type,எங்களை பற்றி,"admin.page_list.common.name_tamil.input"
 100.Click the Submit button,click,,"web.global.action.submit.button"
 101.wait for loading,wait,5000,</t>
+  </si>
+  <si>
+    <t>1. Click the dashboard,Click,,"web.global.menu.dashboard"
+2. Click the setting menu,click,"admin.setting.sidebar.menu"
+3. Click the site setting menu,click,"admin.setting.site_setting.sidebar_menu"
+4. Click in clear (X),click,,"admin.settings.btn_clear_driver_algorithm"
+5. Click on driver algorithm,click,,"admin.settings.dropdown_driver_algorithm"
+6. Click the competitive algorithm,click,,"admin.setting.site_settings.driver_algorithm.competitive_algorithm"
+7. Enter 180 seconds,type,180,"admin.settings.input_user_request_timeout"
+8. Click in clear (X),click,,"admin.settings.btn_clear_calculation_method"
+9. wait for,wait,1000
+10. Click the calculate method,click,,"admin.settings.dropdown_calculation_method"
+11. Click the find distance/eta,click,,"admin.setting.site_settings.calculation_for_transport_service.calculation_method"
+12. Click in clear (X),click,,"admin.settings.btn_clear_google_login"
+13. Click the dropdown google,click,,"admin.settings.btn_trigger_google_login"
+14. Click the google ON,click,,"admin.setting.site_settings.social_login.google_login.on"
+15. Click in clear (X),click,,"admin.global.form.btn_clear_provider_subscription"
+16. Click the dropdown driver subscrption,click,,"admin.global.form.btn_trigger_driver_subscription"
+17. Click subscrption button ON,click,,"admin.global.form.dropdown_option_driver_subscription_on"
+18. Click in clear (X),click,,"admin.global.form.btn_clear_cash"
+19. Click the dropdown cash,click,,"admin.global.form.btn_trigger_cash"
+20. Click cash button ON,click,,"admin.setting.site_settings.payments_method.cash.on"
+21.  Click in clear (X),click,,"admin.global.form.btn_clear_wallet"
+22. Click the dropdown wallet,click,,"admin.global.form.btn_trigger_wallet"
+23. Click wallet button ON,click,,"admin.setting.site_settings.wallet.on"
+24.Click Auto Settle Dropdown,click,,"admin.setting.site_settings.auto_settle_module.dropdown"
+25.Select Auto Settle Off,click,,"admin.setting.site_settings.auto_settle_module.off"
+26. Click in clear (X),click,,"admin.settings.Driver_approval.btn_clear_change_algorithm"
+27. Click the Dropdown,click,,"admin.settings.Driver_approval.btn_trigger_change_algorithm"
+28. Click Driver Approval,click,,"admin.setting.site_settings.account_manual_approvel"
+29. Click in clear (X),click,,"admin.settings.document.btn_clear_change_algorithm"
+30. Click the Dropdown,click,,"admin.settings.document.btn_trigger_change_algorithm"
+31. Click Approval Document,click,,"admin.setting.site_settings.document_manual_approvel"
+32.Click the Dropdown,click,,"admin.settings.document._email_notification_dropdown"
+33.Click On Option,click,,"admin.settings.document._email_notification_option_on"
+34.Click the submit,click,,"admin.settings.btn_submit"
+35.Wait For Submit,wait,2000,</t>
   </si>
 </sst>
 </file>
@@ -2104,7 +2106,7 @@
         <v>75</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2204,7 +2206,7 @@
         <v>83</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2302,7 +2304,7 @@
         <v>88</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2371,36 +2373,36 @@
         <v>2</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>110</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="F2" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -2488,7 +2490,7 @@
         <v>24</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2583,16 +2585,16 @@
         <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2681,16 +2683,16 @@
         <v>37</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2782,7 +2784,7 @@
         <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2877,10 +2879,10 @@
         <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2975,16 +2977,16 @@
         <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -3171,10 +3173,10 @@
         <v>68</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
106th Commit: Epic Five Created And Initiated
</commit_message>
<xml_diff>
--- a/EPIC_0001_Platform_Configuration.xlsx
+++ b/EPIC_0001_Platform_Configuration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E67BB8-CAC1-47BD-BA87-21E8185578DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AAA07C-FCF9-42CD-A533-7B886990B80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>

</xml_diff>

<commit_message>
112th Commit: Epic Six Completed And Epic One Updated
</commit_message>
<xml_diff>
--- a/EPIC_0001_Platform_Configuration.xlsx
+++ b/EPIC_0001_Platform_Configuration.xlsx
@@ -8,24 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AAA07C-FCF9-42CD-A533-7B886990B80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942F1953-C283-44D1-865F-21E1DDEB9E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
     <sheet name="Site_Setting" sheetId="48" r:id="rId2"/>
     <sheet name="City_Area" sheetId="61" r:id="rId3"/>
-    <sheet name="Geo_Fencing" sheetId="62" r:id="rId4"/>
-    <sheet name="Page_List" sheetId="63" r:id="rId5"/>
-    <sheet name="App_Settings" sheetId="64" r:id="rId6"/>
-    <sheet name="Panic_Call" sheetId="65" r:id="rId7"/>
-    <sheet name="Report_Issues" sheetId="66" r:id="rId8"/>
-    <sheet name="Add_Category" sheetId="67" r:id="rId9"/>
-    <sheet name="Add_Vehicle_Type" sheetId="68" r:id="rId10"/>
-    <sheet name="Required_Documents" sheetId="70" r:id="rId11"/>
-    <sheet name="Service_Settings" sheetId="71" r:id="rId12"/>
-    <sheet name="DataCleanUpSheet" sheetId="72" r:id="rId13"/>
+    <sheet name="City_Admin" sheetId="73" r:id="rId4"/>
+    <sheet name="Geo_Fencing" sheetId="62" r:id="rId5"/>
+    <sheet name="Page_List" sheetId="63" r:id="rId6"/>
+    <sheet name="App_Settings" sheetId="64" r:id="rId7"/>
+    <sheet name="Panic_Call" sheetId="65" r:id="rId8"/>
+    <sheet name="Report_Issues" sheetId="66" r:id="rId9"/>
+    <sheet name="Add_Category" sheetId="67" r:id="rId10"/>
+    <sheet name="Add_Vehicle_Type" sheetId="68" r:id="rId11"/>
+    <sheet name="Required_Documents" sheetId="70" r:id="rId12"/>
+    <sheet name="Service_Settings" sheetId="71" r:id="rId13"/>
+    <sheet name="DataCleanUpSheet" sheetId="72" r:id="rId14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="131">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -385,9 +386,6 @@
     <t>TC_GF_561</t>
   </si>
   <si>
-    <t>TC_RG_04_Geo_Fencing</t>
-  </si>
-  <si>
     <t>Add a new restricted area and edit it with new name, location in Admin Web</t>
   </si>
   <si>
@@ -399,9 +397,6 @@
   </si>
   <si>
     <t>CF_TC_680</t>
-  </si>
-  <si>
-    <t>TC_RG_05_Page_List</t>
   </si>
   <si>
     <t>Verify the admin can update all Customer App Support and Driver App Support pages successfully in a single end-to-end flow.</t>
@@ -522,9 +517,6 @@
     <t>Verify the admin can manage Home Page Slider and Source Overview successfully</t>
   </si>
   <si>
-    <t>TC_RG_06_App_Settings</t>
-  </si>
-  <si>
     <t>Admin Web user is logged in and App Settings module is accessible</t>
   </si>
   <si>
@@ -536,9 +528,6 @@
   </si>
   <si>
     <t>Verify the admin can add a new Panic Call record and search the created record successfully in a single end-to-end flow.</t>
-  </si>
-  <si>
-    <t>TC_RG_07_Panic_Call</t>
   </si>
   <si>
     <t>CF_TC_651</t>
@@ -597,17 +586,11 @@
     <t>CF_TC_655</t>
   </si>
   <si>
-    <t>TC_RG_08_Report_Issues</t>
-  </si>
-  <si>
     <t xml:space="preserve">SA_RI_03
 </t>
   </si>
   <si>
     <t>TC_TS_30</t>
-  </si>
-  <si>
-    <t>TC_RG_09_Add_Category</t>
   </si>
   <si>
     <t>Transport Services - Add Transport Category</t>
@@ -702,9 +685,6 @@
   </si>
   <si>
     <t>Verify the admin can add a new Vehicle Type successfully.</t>
-  </si>
-  <si>
-    <t>TC_RG_10_Add_Vehicle_Type</t>
   </si>
   <si>
     <t>1. Click Dashboard Icon.
@@ -796,9 +776,6 @@
     <t>Admin Web user is logged in, Transport Services module is accessible, and a Transport Service is already available.</t>
   </si>
   <si>
-    <t>TC_RG_11_Required_Documents</t>
-  </si>
-  <si>
     <t xml:space="preserve">SA_RI_15
 </t>
   </si>
@@ -838,9 +815,6 @@
   </si>
   <si>
     <t>TC_RD_117</t>
-  </si>
-  <si>
-    <t>TC_RG_12_Service_Settings</t>
   </si>
   <si>
     <t xml:space="preserve">SA_RI_16
@@ -901,54 +875,6 @@
 24.Click Deactive Button,click,,"web.global.report_issue.faq.deactivate.button"
 25.Click Active Button,click,,"web.global.report_issue.faq.activate.button"
 26.wait for popup,wait,2000,</t>
-  </si>
-  <si>
-    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-2. Click Setting menu,click,,"web.global.menu.settings"
-3. Click City area menu,click,,"admin.menu.city_area"
-4. Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
-5. Click Add City Area button,click,,"admin.city_area.btn_add"
-6. Wait For City Area heading,wait_until_visible,,"admin.city_area.add_heading"
-7. Enter Area Name,type,triplicane_{timestamp} &gt;&gt; areaName,"admin.city_area.input_name"
-8. Open Status Dropdown,click,,"admin.city_area.dropdown_status"
-9. Select Active,click,,"admin.city_area.select_status_active"
-10. Enter City Area,type,triplicane,"admin.city_area.input_search_location"
-11. wait,1000,,
-12. Select First Option,arrow_down,,"admin.city_area.input_search_location"
-13. Confirm Option,press_enter,,"admin.city_area.input_search_location"
-14. wait,1000,,
-15. Map Polygon,draw polygon,"-60;-60 : 60;-60 : 60;60 : -60;60","//div[@class='ol-layer']//canvas"
-16. Click Submit,click,,"web.global.action.submit"
-17. Wait For Success Message,wait_until_visible,,"web.global.toast.success"
-18. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-19. Click Transport Services,click,,"admin.transport.menu.card"
-20. Wait For Transport Page,wait_until_visible,,"admin.transport.page.header"
-21. Click Add Category,click,,"admin.transport.add_category.btn"
-22. Open Select City Dropdown,click,,"admin.transport.city.dropdown"
-23. Search City Area,type,{areaName},"admin.transport.input_filter_city"
-24. Verify Area in Dropdown,verify,,"admin.transport.city.dynamic_option"
-25. Click close,click,,"web.global.action.close"
-26. wait for data,wait,2000,
-27.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-28. Click Setting menu,click,,"web.global.menu.settings"
-29. Click City admin menu,click,,"admin.menu.city_admin"
-30. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
-31. Click Add City Admin button,click,,"admin.city_admin.btn_add"
-32. Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
-33. Select {areaName},click,,"admin.city_admin.select_dynamic_option"
-34. Verify Selection,verify,,"admin.city_admin.verify_dropdown_value"
-35.Wait For Verify,wait,2000,
-36.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-37.Click Setting menu,click,,"web.global.menu.settings"
-38.Click City area menu,click,,"admin.menu.city_area"
-39.Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
-40.Serch Created Area,type,{areaName},"admin.city_area.area_filter_input"
-41.Wait For Load,wait,1000,
-42.Click City Area Edit,click,,"admin.city_area.edit_button"
-43.Open Status Dropdown,click,,"admin.city_area.dropdown_active_status"
-44.Select Inactive,click,,"admin.city_area.select_status_inactive"
-45.Click Submit,click,,"web.global.action.submit"
-46.Wait For Submit,2000,</t>
   </si>
   <si>
     <t>1. Log into the Super Admin Web Portal and click the Dashboard Icon on the sidebar menu.
@@ -1101,24 +1027,6 @@
 </t>
   </si>
   <si>
-    <t>1. Click Dashboard,Click,,"web.global.menu.dashboard"
-2. Click Setting,click,,"admin.setting.sidebar.menu"
-3. Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
-4. Click Add panic call button,click,,"admin.setting.panic_call.add_btn"
-5. Enter name,type,police_{randomAlpha}&gt;&gt;policeName,"admin.setting.panic_call.name_input"
-6. Enter name in tamil,type,காவல்துறை,"admin.setting.panic_call.tamil_name_input"
-7. Enter name in hindi,type,पुलिस,"admin.setting.panic_call.hindi_name_input"
-8. Contact number,type,{randomPhone},"admin.setting.panic_call.contact_number"
-9. Select Status button,click,,"admin.setting.panic_call.status_dropdown"
-10. Select Active status,click,,"admin.setting.panic_call.activate_status_dropdown"
-11. Submit button,click,,"web.global.action.submit"
-12. Search name,type,{policeName},"admin.setting.panic_call.search_name"
-13.Wait For Load,wait,1000,
-14.Delete Panic Call Delete,click,,"admin.setting.panic_call.delete_btn"
-15.Confirm Delete,click,,"admin.setting.panic_call.confirm_delete_btn"
-16. Wait For Delete,wait,2000,</t>
-  </si>
-  <si>
     <t>1. Click Dashboard.
 2. Click Setting.
 3. Click Panic Call Setting.
@@ -1139,36 +1047,6 @@
 18. Enter created Panic Call Name.
 19. Verify Panic Call record is displayed in the search results.
 20.Delete The Displayed Panic Call</t>
-  </si>
-  <si>
-    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
-2. Click Transports Services Menu,click,, "admin.transport.menu.card"
-3.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
-4.Click  Add Category,click,, "admin.transport.add_category.btn"
-5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "admin.transport.name.input"
-6.Enter Service Name Arabic, type, رحلة بالحافلة, "admin.transport.name_ar.input"
-7.Enter Slug, type, Bus Ride, "admin.transport.slug.input"
-8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "admin.transport.image.file"
-9.wait,2000,,
-10.Open status Dropdown,click,, "admin.transport.status.dropdown"
-11.Select Activate,click,, "admin.transport.status.activate_option"
-12.Open Select City Dropdown,click,, "admin.transport.city.dropdown"
-13.Select City Area,click,,"admin.transport.city.dynamic_option_regression_city_area"
-14.Click  Submit,click,, "web.global.action.submit"
-15.Wait Till Sucess, wait_until_visible, , "web.global.toast.info"
-16.Wait To Load,wait,2000,
-17.Click Dashboard Icon,click,, "web.global.menu.dashboard"
-18.Click Transports Services Menu,click,, "admin.transport.menu.card"
-19.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
-20.Select Transport Service Name,type,{transportName},"admin.transport.grid.name_filter"
-21.Wait For Load,wait,2000,
-22.Click Edit,click,,"admin.transport.edit_btn"
-23.Scroll Transport From,tab,5,"admin.transport.name.input"
-24.Open status Dropdown,click,, "admin.transport.status.dropdown"
-25.Select Deactivate,click,, "admin.transport.status.deactivate_option"
-26.Click  Submit,click,, "web.global.action.submit"
-27.Wait For Update,wait,2000,
-28.Click  back,click,, "admin.transport.back.btn"</t>
   </si>
   <si>
     <t>a new Transport Service category successfully.
@@ -1198,64 +1076,6 @@
 24.Click Submit</t>
   </si>
   <si>
-    <t>1. Click Dashboard Icon,click,, "web.global.menu.dashboard"
-2.Click Transports Services Menu,click,, "admin.transport.menu.card"
-3.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
-4.Click Home Icon ,click,, "admin.transport.home.icon"
-5.Click Settings ,click,, "admin.transport.menu.settings"
-6.Click Vehicle Type,click,, "admin.transport.settings.vehicle_type"
-7.Click Add Vehicle Type,click,, "admin.transport.vehicle.add_type.btn"
-8.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "admin.transport.vehicle.name.input"
-9.Enter Base Fare, type, 150, "admin.transport.vehicle.base_fare.input"
-10.Enter Base Fare Max Kilometer, type, 10, "admin.transport.vehicle.base_km.input"
-11.Open Extra Distance Fare Dropdown,click,, "admin.transport.vehicle.extra_fare_type.dropdown"
-12.Select Amount,click,, "admin.transport.status.amount_option"
-13.Enter Extra Distance Fare , type, 10, "admin.transport.vehicle.extra_fare.input"
-14.Enter Free Waiting Time , type, 10, "admin.transport.vehicle.waiting_free.input"
-15.Open Waiting Charge Dropdown,click,, "admin.transport.vehicle.waiting_type.dropdown"
-16.Select Amount,click,, "admin.transport.status.amount_option"
-17.Enter Waiting Rate , type, 10, "admin.transport.vehicle.waiting_rate.input"
-18.Enter Included Trip Waiting , type, 10, "admin.transport.vehicle.trip_waiting_free.input"
-19.Open Trip Waiting Charge Dropdown,click,, "admin.transport.vehicle.trip_waiting_type.dropdown"
-20.Select Amount,click,, "admin.transport.status.amount_option"
-21.Enter Trip Waiting Rate , type,50, "admin.transport.vehicle.trip_waiting_rate.input"
-22.Enter Free Pickup Distance , type,5, "admin.transport.vehicle.pickup_free.input"
-23.Open Pickup Charge Dropdown,click,, "admin.transport.vehicle.pickup_type.dropdown"
-24.Select Amount,click,, "admin.transport.status.amount_option"
-25.Enter Pickup Fee, type,50, "admin.transport.vehicle.pickup_fee.input"
-26.Open Customer Fee  Dropdown,click,, "admin.transport.vehicle.customer_type.dropdown"
-27.Select Amount,click,, "admin.transport.status.amount_option"
-28.Enter Customer Fee, type,50, "admin.transport.vehicle.customer_fee.input"
-29.Open Customer GST  Dropdown,click,, "admin.transport.vehicle.customer_gst_type.dropdown"
-30.Select Amount,click,, "admin.transport.status.amount_option"
-31.Enter  GST amount, type,50, "admin.transport.vehicle.customer_gst.input"
-32.Open Driver Fee  Dropdown,click,, "admin.transport.vehicle.driver_type.dropdown"
-33.Select Amount,click,, "admin.transport.status.amount_option"
-34.Enter  Driver Fee, type,50, "admin.transport.vehicle.driver_fee.input"
-35.Open Driver GST  Dropdown,click,, "admin.transport.vehicle.driver_gst_type.dropdown"
-36.Select Amount,click,, "admin.transport.status.amount_option"
-37.Enter Driver Gst,type,50, "admin.transport.vehicle.driver_gst.input"
-38.Open Status Dropdown,click,, "admin.transport.vehicle.status.dropdown"
-39.Select Active,click,, "admin.transport.status.active_option"
-40.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "admin.transport.vehicle.image.file"
-41.Enter Notifiacation,type,50, "admin.transport.vehicle.notify_km.input"
-42.Enter Driver Request ETA,type,50, "admin.transport.vehicle.eta_limit.input"
-43.Enter Driver Request KM,type,50, "admin.transport.vehicle.km_limit.input"
-44.Enter Package Idle Free Time,type,30,"admin.transport.vehicle.package_idle_free_time"
-45.Enter Package Idle Time Fee,type,50,"admin.transport.vehicle.package_idle_time_fee"
-46.Open Night Charge Timing Status Dropdown,click,, "admin.transport.night.status.dropdown"
-47.Select Active,click,, "admin.transport.status.active_option"
-48.Click Surcharge Time Checkbox, click, , "admin.transport.night.everyday.checkbox"
-49.Enter From Time, type, 100000AM, "admin.transport.night.from_time.input"
-50.Enter To Time, type, 220000PM, "admin.transport.night.to_time.input"
-51.Open  Dropdown,click,, "admin.transport.night.type.dropdown"
-52.Select Amount,click,, "admin.transport.status.amount_option"
-53.Enter  Price, type,50, "admin.transport.night.price.input"
-54.Click  Submit,click,, "web.global.action.submit"
-55.Wait For Sucess,wait_until_visible, , "web.global.toast.info"
-56.Wait For Popup,wait,3000,</t>
-  </si>
-  <si>
     <t>1.Click Dashboard,Click,,"web.global.menu.dashboard"
 2.Click Transport Service,Click,,"admin.transport.menu.card"
 3.Click Search Box,click,,"admin.transport.search.input_box"
@@ -1421,20 +1241,10 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
-2.Remove  Document Created,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
-3..Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
-4.Remove  Transport Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
-</t>
-  </si>
-  <si>
     <t>SA_TS_XX</t>
   </si>
   <si>
     <t>Clean The Test Data Created During Test Run Of Epic One</t>
-  </si>
-  <si>
-    <t>TC_RG_13_test_data_cleanup</t>
   </si>
   <si>
     <t>No Manual Test Cases Since this is a data cleanup sheet after test execution of epic one</t>
@@ -1578,6 +1388,390 @@
 33.Click On Option,click,,"admin.settings.document._email_notification_option_on"
 34.Click the submit,click,,"admin.settings.btn_submit"
 35.Wait For Submit,wait,2000,</t>
+  </si>
+  <si>
+    <t>Removed Test Cases</t>
+  </si>
+  <si>
+    <t>SA_RD_03</t>
+  </si>
+  <si>
+    <t>CityAdmin</t>
+  </si>
+  <si>
+    <t>TC_SA_03_add_city_admin</t>
+  </si>
+  <si>
+    <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Setting menu,click,,"web.global.menu.settings"
+3. Click City admin menu,click,,"admin.menu.city_admin"
+4. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
+5. Click Add City Admin button,click,,"admin.city_admin.btn_add"
+6. Wait For Admin heading,wait_until_visible,,"admin.city_admin.add_heading"
+7.Select Name field,click,,"admin.city_admin.input_name"
+8. Enter Admin Name,type,faizal{randomAlpha} &gt;&gt; adminName,"admin.city_admin.input_name"
+9.Select Email field,click,,"admin.city_admin.input_email"
+10. Enter Email,type,faizal_{timestamp}@gmail.com,"admin.city_admin.input_email"
+11.select the password field,click,,"admin.city_admin.input_password"
+12.Enter the Password as "faizal@123",type,faizal@123,"admin.city_admin.input_password"
+13.Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
+14.Select {areaName},click,,"admin.city_admin.select_dynamic_option"
+15. Click on the "Transport Service" → "Auto Ride" checkbox,click,,"admin.city_admin.chk_transport_auto_ride"
+16.Click on the "Customers" → "Add Customers" checkbox,click,,"admin.city_admin.chk_customer_add"
+17.Click on the "Customers" → "Verified Customers"checkbox,click,,"admin.city_admin.chk_customer_verified"
+18.Click on the "Customers" → "Non Verified Customers" checkbox,click,,"admin.city_admin.chk_customer_unverified"
+19.Click on the "Customers" → "Blocked Customers" checkbox,click,,"admin.city_admin.chk_customer_blocked"
+20.Click on the "Customers" → "Deleted Customers" checkbox,click,,"admin.city_admin.chk_customer_deleted"
+21.Click on the "Providers" → "Transport Providers List" checkbox,click,,"admin.city_admin.chk_provider_list"
+22.Click on the "Drivers" → "Add Driver" checkbox,click,,"admin.city_admin.chk_driver_add"
+23.Click on the "Drivers" → "Approved Drivers" checkbox,click,,"admin.city_admin.chk_driver_approved"
+24.Click on the "Drivers" → "Un-Approved Drivers" checkbox,click,,"admin.city_admin.chk_driver_unapproved"
+25.Click on the "Drivers" → "Blocked Drivers" checkbox,click,,"admin.city_admin.chk_driver_blocked"
+26.Click on the "Drivers" → "Reject Drivers" checkbox,click,,"admin.city_admin.chk_driver_rejected"
+27.Click on the "Drivers" → "Deleted Drivers" checkbox,click,,"admin.city_admin.chk_driver_deleted"
+28.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox,click,,"admin.city_admin.chk_subscription_plan"
+29.Click on the "Cash Out" → "Driver Cash Out" checkbox,click,,"admin.city_admin.chk_cashout"
+30.Click on the "Report Issue" → "Customer Report Issues" checkbox,click,,"admin.city_admin.chk_report_customer"
+31.Click on the "Report Issue" → "Driver Report Issues" checkbox,click,,"admin.city_admin.chk_report_driver"
+32.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"admin.city_admin.chk_report_provider"
+33.Click on the "Report Issue" → "Report issue settings" checkbox,click,,"admin.city_admin.chk_report_settings"
+34.Click on the "Report Issue" → "FAQs" checkbox,click,,"admin.city_admin.chk_report_faqs"
+35.Click Submit,click,,"web.global.login.submit_btn"
+36. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
+37.Filter admin name,type,{adminName},"admin.city_admin.input_name_filter"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
+RunSheet: AddCityArea</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>System State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
+    </r>
+  </si>
+  <si>
+    <t>21.Click on the "Customers" → "Pending Customers" checkbox,click,,admin.city_admin.chk_customer_pending
+35.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox,click,,admin.city_admin.chk_web_header_footer
+36.Click on the "Website Settings" → "Home Page Settings" checkbox,click,,admin.city_admin.chk_web_homepage
+37.Click on the "Website Settings" → "Delivery Settings" checkbox,click,,admin.city_admin.chk_web_delivery
+38.Click on the "Website Settings" → "Transport Settings" checkbox,click,,admin.city_admin.chk_web_transport
+39.Click on the "Website Settings" → "FAQs" checkbox,click,,admin.city_admin.chk_web_faqs</t>
+  </si>
+  <si>
+    <t>TC_RG_04_add_city_admin</t>
+  </si>
+  <si>
+    <t>1. Click on "Dashboard" from the navigation menu.
+2. Click on "Settings" in the navigation menu.
+3. Click on "City Admin" from the sidebar menu.
+4. Wait for the City Admin List heading to display on screen.
+5. Click the "Add City Admin" button.
+6. Wait for the Add City Admin page heading to display.
+7. Click the Name input field.
+8. Enter a dynamic admin name (faizal{randomAlpha}) into the Name field.
+9. Click the Email input field.
+10. Enter a dynamic email address (faizal_{timestamp}@gmail.com) into the Email field.
+11. Click the Password input field.
+12. Enter the password ("faizal@123") into the Password field.
+13. Open the Select City dropdown.
+14. Select the target area/city ({areaName}) from the dropdown options.
+15. Select the checkbox for "Transport Service" → "Auto Ride" permission.
+16. Select the checkbox for "Customers" → "Add Customers" permission.
+17. Select the checkbox for "Customers" → "Verified Customers" permission.
+18. Select the checkbox for "Customers" → "Non Verified Customers" permission.
+19. Select the checkbox for "Customers" → "Blocked Customers" permission.
+20. Select the checkbox for "Customers" → "Deleted Customers" permission.
+21. Select the checkbox for "Providers" → "Transport Providers List" permission.
+22. Select the checkbox for "Drivers" → "Add Driver" permission.
+23. Select the checkbox for "Drivers" → "Approved Drivers" permission.
+24. Select the checkbox for "Drivers" → "Un-Approved Drivers" permission.
+25. Select the checkbox for "Drivers" → "Blocked Drivers" permission.
+26. Select the checkbox for "Drivers" → "Reject Drivers" permission.
+27. Select the checkbox for "Drivers" → "Deleted Drivers" permission.
+28. Select the checkbox for "Subscription Plan" → "Driver Subscription Plan" permission.
+29. Select the checkbox for "Cash Out" → "Driver Cash Out" permission.
+30. Select the checkbox for "Report Issue" → "Customer Report Issues" permission.
+31. Select the checkbox for "Report Issue" → "Driver Report Issues" permission.
+32. Select the checkbox for "Report Issue" → "Provider Report Issues" permission.
+33. Select the checkbox for "Report Issue" → "Report issue settings" permission.
+34. Select the checkbox for "Report Issue" → "FAQs" permission.
+35. Click the "Submit" button to save the new City Admin profile.
+36. Wait for the success toast notification message to display.
+37. Filter the City Admin list using the newly created admin name to verify creation.</t>
+  </si>
+  <si>
+    <t>TC_RG_05_Geo_Fencing</t>
+  </si>
+  <si>
+    <t>TC_RG_06_Page_List</t>
+  </si>
+  <si>
+    <t>TC_RG_07_App_Settings</t>
+  </si>
+  <si>
+    <t>TC_RG_08_Panic_Call</t>
+  </si>
+  <si>
+    <t>TC_RG_09_Report_Issues</t>
+  </si>
+  <si>
+    <t>TC_RG_10_Add_Category</t>
+  </si>
+  <si>
+    <t>TC_RG_11_Add_Vehicle_Type</t>
+  </si>
+  <si>
+    <t>TC_RG_12_Required_Documents</t>
+  </si>
+  <si>
+    <t>TC_RG_13_Service_Settings</t>
+  </si>
+  <si>
+    <t>TC_RG_14_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>1.Remove Test Area,sql delete,,"DELETE FROM we1.admin_area_list WHERE name = '{areaName}';"
+2.Remove  Document Created,sql delete,,"DELETE FROM we1.required_documents WHERE name = '{documentName}';"
+3..Remove Bus Vehicle Variation Volvo,sql delete,,"DELETE FROM we1.transport_vehicle_type WHERE name = '{busTypeName}';"
+4.Remove  Transport Service,sql delete,,"DELETE FROM we1.service_category WHERE name = '{transportName}';"
+5.Remove City Admin,sql delete,,"DELETE FROM we1.super_admin WHERE name = '{adminName}';"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Setting menu,click,,"web.global.menu.settings"
+3. Click City area menu,click,,"admin.menu.city_area"
+4. Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
+5. Click Add City Area button,click,,"admin.city_area.btn_add"
+6. Wait For City Area heading,wait_until_visible,,"admin.city_area.add_heading"
+7. Enter Area Name,type,triplicane_{timestamp} &gt;&gt; areaName,"admin.city_area.input_name"
+8. Open Status Dropdown,click,,"admin.city_area.dropdown_status"
+9. Select Active,click,,"admin.city_area.select_status_active"
+10. Enter City Area,type,triplicane,"admin.city_area.input_search_location"
+11. wait,1000,,
+12. Select First Option,arrow_down,,"admin.city_area.input_search_location"
+13. Confirm Option,press_enter,,"admin.city_area.input_search_location"
+14. wait,1000,,
+15. Map Polygon,draw polygon,"-60;-60 : 60;-60 : 60;60 : -60;60","//div[@class='ol-layer']//canvas"
+16. Click Submit,click,,"web.global.action.submit"
+17. Wait For Success Message,wait_until_visible,,"web.global.toast.success"
+18. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+19. Click Transport Services,click,,"admin.transport.menu.card"
+20. Wait For Transport Page,wait_until_visible,,"admin.transport.page.header"
+21. Click Add Category,click,,"admin.transport.add_category.btn"
+22. Open Select City Dropdown,click,,"admin.transport.city.dropdown"
+23. Search City Area,type,{areaName},"admin.transport.input_filter_city"
+24. Verify Area in Dropdown,verify,,"admin.transport.city.dynamic_option"
+25. Click close,click,,"web.global.action.close"
+26. wait for data,wait,2000,
+27.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+28. Click Setting menu,click,,"web.global.menu.settings"
+29. Click City admin menu,click,,"admin.menu.city_admin"
+30. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
+31. Click Add City Admin button,click,,"admin.city_admin.btn_add"
+32. Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
+33. Select {areaName},click,,"admin.city_admin.select_dynamic_option"
+34. Verify Selection,verify,,"admin.city_admin.verify_dropdown_value"
+35.Wait For Verify,wait,2000,
+36.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+37.Click Setting menu,click,,"web.global.menu.settings"
+38.Click City area menu,click,,"admin.menu.city_area"
+39.Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
+40.Serch Created Area,type,{areaName},"admin.city_area.area_filter_input"
+43.Wait For Load,wait,1000,
+</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard,Click,,"web.global.menu.dashboard"
+2. Click Setting,click,,"admin.setting.sidebar.menu"
+3. Click Panic call setting,click,,"admin.setting.panic_call.sidebar_menu"
+4. Click Add panic call button,click,,"admin.setting.panic_call.add_btn"
+5. Enter name,type,police_{randomAlpha}&gt;&gt;policeName,"admin.setting.panic_call.name_input"
+6. Enter name in tamil,type,காவல்துறை,"admin.setting.panic_call.tamil_name_input"
+7. Enter name in hindi,type,पुलिस,"admin.setting.panic_call.hindi_name_input"
+8. Contact number,type,120,"admin.setting.panic_call.contact_number"
+9. Select Status button,click,,"admin.setting.panic_call.status_dropdown"
+10. Select Active status,click,,"admin.setting.panic_call.activate_status_dropdown"
+11. Submit button,click,,"web.global.action.submit"
+12. Search name,type,{policeName},"admin.setting.panic_call.search_name"
+13.Wait For Load,wait,1000,
+14.Delete Panic Call Delete,click,,"admin.setting.panic_call.delete_btn"
+15.Confirm Delete,click,,"admin.setting.panic_call.confirm_delete_btn"
+16. Wait For Delete,wait,2000,</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2.Click Transports Services Menu,click,, "admin.transport.menu.card"
+3.Filter Services List,type,{transportName}, "admin.transport.grid.name_filter"
+4.Click Home Icon ,click,, "admin.transport.home.icon"
+5.Click Settings ,click,, "admin.transport.menu.settings"
+6.Click Vehicle Type,click,, "admin.transport.settings.vehicle_type"
+7.Click Add Vehicle Type,click,, "admin.transport.vehicle.add_type.btn"
+8.Enter Vehicle Type Name, type, volvo{randomAlpha}&gt;&gt;busTypeName, "admin.transport.vehicle.name.input"
+9.Enter Base Fare, type, 150, "admin.transport.vehicle.base_fare.input"
+10.Enter Base Fare Max Kilometer, type, 10, "admin.transport.vehicle.base_km.input"
+11.Open Extra Distance Fare Dropdown,click,, "admin.transport.vehicle.extra_fare_type.dropdown"
+12.Select Amount,click,, "admin.transport.status.amount_option"
+13.Enter Extra Distance Fare , type, 10, "admin.transport.vehicle.extra_fare.input"
+14.Enter Free Waiting Time , type, 10, "admin.transport.vehicle.waiting_free.input"
+15.Open Waiting Charge Dropdown,click,, "admin.transport.vehicle.waiting_type.dropdown"
+16.Select Amount,click,, "admin.transport.status.amount_option"
+17.Enter Waiting Rate , type, 10, "admin.transport.vehicle.waiting_rate.input"
+18.Enter Included Trip Waiting , type, 10, "admin.transport.vehicle.trip_waiting_free.input"
+19.Open Trip Waiting Charge Dropdown,click,, "admin.transport.vehicle.trip_waiting_type.dropdown"
+20.Select Amount,click,, "admin.transport.status.amount_option"
+21.Enter Trip Waiting Rate , type,50, "admin.transport.vehicle.trip_waiting_rate.input"
+22.Enter Free Pickup Distance , type,5, "admin.transport.vehicle.pickup_free.input"
+23.Open Pickup Charge Dropdown,click,, "admin.transport.vehicle.pickup_type.dropdown"
+24.Select Amount,click,, "admin.transport.status.amount_option"
+25.Enter Pickup Fee, type,50, "admin.transport.vehicle.pickup_fee.input"
+26.Open Customer Fee  Dropdown,click,, "admin.transport.vehicle.customer_type.dropdown"
+27.Select Amount,click,, "admin.transport.status.amount_option"
+28.Enter Customer Fee, type,50, "admin.transport.vehicle.customer_fee.input"
+29.Open Customer GST  Dropdown,click,, "admin.transport.vehicle.customer_gst_type.dropdown"
+30.Select Amount,click,, "admin.transport.status.amount_option"
+31.Enter  GST amount, type,50, "admin.transport.vehicle.customer_gst.input"
+32.Open Driver Fee  Dropdown,click,, "admin.transport.vehicle.driver_type.dropdown"
+33.Select Amount,click,, "admin.transport.status.amount_option"
+34.Enter  Driver Fee, type,50, "admin.transport.vehicle.driver_fee.input"
+35.Open Driver GST  Dropdown,click,, "admin.transport.vehicle.driver_gst_type.dropdown"
+36.Select Amount,click,, "admin.transport.status.amount_option"
+37.Enter Driver Gst,type,50, "admin.transport.vehicle.driver_gst.input"
+38.Open Status Dropdown,click,, "admin.transport.vehicle.status.dropdown"
+39.Select Active,click,, "admin.transport.status.active_option"
+40.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/volvo.jpg", "admin.transport.vehicle.image.file"
+41.Enter Notifiacation,type,50, "admin.transport.vehicle.notify_km.input"
+42.Enter Driver Request ETA,type,50, "admin.transport.vehicle.eta_limit.input"
+43.Enter Driver Request KM,type,50, "admin.transport.vehicle.km_limit.input"
+44.Enter PickUp Arrival Enable Button,type,50,"admin.transport.pickup_arrival.Enable_btn"
+45.Enter PickUp Arrival Show Notification,type,50,"admin.transport.pickup_arrival.show_notification"
+46.Enter Package Idle Free Time,type,30,"admin.transport.vehicle.package_idle_free_time"
+47.Enter Package Idle Time Fee,type,50,"admin.transport.vehicle.package_idle_time_fee"
+48.Open Night Charge Timing Status Dropdown,click,, "admin.transport.night.status.dropdown"
+49.Select Active,click,, "admin.transport.status.active_option"
+50.Click Surcharge Time Checkbox, click, , "admin.transport.night.everyday.checkbox"
+51.Enter From Time, type, 100000AM, "admin.transport.night.from_time.input"
+52.Enter To Time, type, 220000PM, "admin.transport.night.to_time.input"
+53.Open  Dropdown,click,, "admin.transport.night.type.dropdown"
+54.Select Amount,click,, "admin.transport.status.amount_option"
+55.Enter  Price, type,50, "admin.transport.night.price.input"
+56.Click  Submit,click,, "web.global.action.submit"
+57.Wait For Sucess,wait_until_visible, , "web.global.toast.info"
+58.Wait For Popup,wait,3000,</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+2. Click Transports Services Menu,click,, "admin.transport.menu.card"
+3.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+4.Click  Add Category,click,, "admin.transport.add_category.btn"
+5.Enter Service Name, type, Bus Ride{randomAlpha}&gt;&gt;transportName, "admin.transport.name.input"
+6.Enter Service Name Arabic, type, رحلة بالحافلة, "admin.transport.name_ar.input"
+7.Enter Slug, type, Bus Ride, "admin.transport.slug.input"
+8.Upload Transport Service Image, uploadfile, "src/main/resources/test-data/bus.jpg", "admin.transport.image.file"
+9.wait,2000,,
+10.Open status Dropdown,click,, "admin.transport.status.dropdown"
+11.Select Activate,click,, "admin.transport.status.activate_option"
+12.Open Select City Dropdown,click,, "admin.transport.city.dropdown"
+13.Select City Area,click,,"admin.transport.city.dynamic_option_regression_city_area"
+14.Click  Submit,click,, "web.global.action.submit"
+15.Wait Till Sucess, wait_until_visible, , "web.global.toast.info"
+16.Wait To Load,wait,2000,
+17.Click Dashboard Icon,click,, "web.global.menu.dashboard"
+18.Click Transports Services Menu,click,, "admin.transport.menu.card"
+19.Wait For Transport Services, wait_until_visible,, "admin.transport.page.header"
+20.Select Transport Service Name,type,{transportName},"admin.transport.grid.name_filter"
+21.Wait For Load,wait,2000,
+22.Click Edit,click,,"admin.transport.edit_btn"
+23.Wait To Load,wait,4000
+24.Scroll Transport From,tab,5,"admin.transport.name.input"
+25.Open status Dropdown,click,, "admin.transport.status.dropdown"
+26.Select Deactivate,click,, "admin.transport.status.deactivate_option"
+27.Click  Submit,click,, "web.global.action.submit"
+28.Wait For Update,wait,2000,
+29.Click  back,click,, "admin.transport.back.btn"</t>
   </si>
 </sst>
 </file>
@@ -2038,6 +2232,104 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4942C78B-FF97-4FA7-A00D-96E4414492E5}">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.44140625" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="45.77734375" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4ED500-CE8C-43B5-A09A-34CB6FB43B13}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2088,34 +2380,34 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>74</v>
+        <v>122</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -2137,7 +2429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29CA9951-BCDC-45CA-B90F-449E473475A9}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2188,31 +2480,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2235,7 +2527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89D43021-0089-49EC-B3A1-EEDBD29B5F98}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2286,31 +2578,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>85</v>
+        <v>124</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2333,7 +2625,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F212A7B3-E2B5-43F7-B627-2EE6125B3067}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2373,36 +2665,36 @@
         <v>2</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -2490,7 +2782,7 @@
         <v>24</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -2579,22 +2871,22 @@
         <v>31</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2618,6 +2910,87 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6326142B-D56E-4616-9248-20BFDCFED237}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="2" max="3" width="19.88671875" customWidth="1"/>
+    <col min="4" max="4" width="25.44140625" customWidth="1"/>
+    <col min="5" max="5" width="34.77734375" customWidth="1"/>
+    <col min="6" max="6" width="38.77734375" customWidth="1"/>
+    <col min="7" max="7" width="64" customWidth="1"/>
+    <col min="8" max="8" width="32.6640625" customWidth="1"/>
+    <col min="9" max="9" width="44.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96A868FA-567D-4204-869D-D8B90B0E6866}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2677,22 +3050,22 @@
         <v>35</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2715,7 +3088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90E9C175-F7EE-471C-B25F-DE0EEBC7429E}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2766,31 +3139,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2813,7 +3186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03961736-D7B8-454D-BD4B-BDA77EE2090B}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2864,31 +3237,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -2911,7 +3284,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A076069-20AA-44BC-B1C2-4ECA85C3527C}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2962,31 +3335,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>119</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -3009,7 +3382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FEFE97B-9A07-41DD-A650-686ECAC76492}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3060,31 +3433,31 @@
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -3105,102 +3478,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4942C78B-FF97-4FA7-A00D-96E4414492E5}">
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.44140625" customWidth="1"/>
-    <col min="4" max="4" width="28.77734375" customWidth="1"/>
-    <col min="5" max="5" width="29.109375" customWidth="1"/>
-    <col min="6" max="6" width="45.77734375" customWidth="1"/>
-    <col min="7" max="7" width="71.44140625" customWidth="1"/>
-    <col min="8" max="8" width="40.44140625" customWidth="1"/>
-    <col min="9" max="9" width="61.88671875" customWidth="1"/>
-    <col min="10" max="10" width="32.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>